<commit_message>
Fix XLSX translations: history sheets, lore text, broken translations
- All 7 history sheets rewritten with proper English (89 entries)
- Codex: 316 lore cells reverted to Korean original (monster/character descriptions)
- Records: 443 lore cells reverted to Korean (adventure journal stories, constellation stories)
- Fixed 355 broken translation cells (repeated words, gibberish)
- Fixed "can" → "Sumin Ban", "김평직" → "Pyeongjik Kim" author names
- Added lore notes: "narrative text kept in original Korean"

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QuestGuide_DesignDocument.xlsx
+++ b/docs/QuestGuide_DesignDocument.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <name val="맑은 고딕"/>
       <charset val="129"/>
@@ -130,6 +130,15 @@
       <color theme="1"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -683,7 +692,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -841,6 +850,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="42" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1505,21 +1541,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L42"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="4.375" customWidth="1" style="32" min="1" max="1"/>
-    <col width="9" customWidth="1" style="32" min="2" max="2"/>
-    <col width="11" customWidth="1" style="32" min="3" max="3"/>
-    <col width="9" customWidth="1" style="32" min="4" max="15"/>
+    <col width="8" customWidth="1" style="32" min="2" max="2"/>
+    <col width="12" customWidth="1" style="32" min="3" max="3"/>
+    <col width="75" customWidth="1" style="32" min="4" max="15"/>
+    <col width="18" customWidth="1" style="46" min="12" max="12"/>
     <col width="11.375" bestFit="1" customWidth="1" style="32" min="16" max="16"/>
     <col width="9" customWidth="1" style="32" min="17" max="16384"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Document History : Quest Guide when </t>
+    <row r="1"/>
+    <row r="2" ht="22" customHeight="1" s="46">
+      <c r="B2" s="61" t="inlineStr">
+        <is>
+          <t>Document History : Quest Guide System</t>
         </is>
       </c>
       <c r="C2" s="5" t="n"/>
@@ -1533,10 +1571,22 @@
       <c r="K2" s="5" t="n"/>
       <c r="L2" s="5" t="n"/>
     </row>
-    <row r="3">
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
+    <row r="3" ht="18" customHeight="1" s="46">
+      <c r="B3" s="62" t="inlineStr">
+        <is>
+          <t>Index</t>
+        </is>
+      </c>
+      <c r="C3" s="62" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D3" s="62" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
       <c r="E3" s="6" t="n"/>
       <c r="F3" s="6" t="n"/>
       <c r="G3" s="6" t="n"/>
@@ -1544,61 +1594,49 @@
       <c r="I3" s="6" t="n"/>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
-      <c r="L3" s="6" t="n"/>
-    </row>
-    <row r="4" ht="22.5" customHeight="1" s="46">
+      <c r="L3" s="62" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="46">
       <c r="A4" s="7" t="n"/>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>Index</t>
-        </is>
-      </c>
-      <c r="C4" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Date</t>
-        </is>
-      </c>
-      <c r="D4" s="33" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="E4" s="47" t="n"/>
-      <c r="F4" s="47" t="n"/>
-      <c r="G4" s="47" t="n"/>
-      <c r="H4" s="47" t="n"/>
-      <c r="I4" s="47" t="n"/>
-      <c r="J4" s="47" t="n"/>
-      <c r="K4" s="48" t="n"/>
-      <c r="L4" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+      <c r="B4" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="64" t="inlineStr">
+        <is>
+          <t>24.05.03</t>
+        </is>
+      </c>
+      <c r="D4" s="64" t="inlineStr">
+        <is>
+          <t>Initial draft</t>
+        </is>
+      </c>
+      <c r="L4" s="65" t="inlineStr">
+        <is>
+          <t>Juwon Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="46">
       <c r="A5" s="30" t="n"/>
-      <c r="B5" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>24.05.03</t>
-        </is>
-      </c>
-      <c r="D5" s="49" t="inlineStr">
-        <is>
-          <t>Initial Draft</t>
-        </is>
-      </c>
-      <c r="E5" s="50" t="n"/>
-      <c r="F5" s="50" t="n"/>
-      <c r="G5" s="50" t="n"/>
-      <c r="H5" s="50" t="n"/>
-      <c r="I5" s="50" t="n"/>
-      <c r="J5" s="50" t="n"/>
-      <c r="K5" s="51" t="n"/>
-      <c r="L5" s="12" t="inlineStr">
+      <c r="B5" s="66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="67" t="inlineStr">
+        <is>
+          <t>25.06.11</t>
+        </is>
+      </c>
+      <c r="D5" s="68" t="inlineStr">
+        <is>
+          <t>UI updated; detailed descriptions added</t>
+        </is>
+      </c>
+      <c r="L5" s="69" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
@@ -1606,283 +1644,95 @@
     </row>
     <row r="6">
       <c r="A6" s="30" t="n"/>
-      <c r="B6" s="31" t="n">
-        <v>2</v>
-      </c>
-      <c r="C6" s="28" t="inlineStr">
-        <is>
-          <t>25.06.11</t>
-        </is>
-      </c>
-      <c r="D6" s="52" t="inlineStr">
-        <is>
-          <t>UI Updated And Description Add</t>
-        </is>
-      </c>
-      <c r="E6" s="53" t="n"/>
-      <c r="F6" s="53" t="n"/>
-      <c r="G6" s="53" t="n"/>
-      <c r="H6" s="53" t="n"/>
-      <c r="I6" s="53" t="n"/>
-      <c r="J6" s="53" t="n"/>
-      <c r="K6" s="54" t="n"/>
-      <c r="L6" s="27" t="inlineStr">
-        <is>
-          <t>Juwon Lee</t>
-        </is>
-      </c>
+      <c r="B6" s="31" t="n"/>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="52" t="n"/>
+      <c r="L6" s="27" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="40" t="n"/>
       <c r="C7" s="40" t="n"/>
       <c r="D7" s="40" t="n"/>
-      <c r="E7" s="55" t="n"/>
-      <c r="F7" s="55" t="n"/>
-      <c r="G7" s="55" t="n"/>
-      <c r="H7" s="55" t="n"/>
-      <c r="I7" s="55" t="n"/>
-      <c r="J7" s="55" t="n"/>
-      <c r="K7" s="56" t="n"/>
       <c r="L7" s="40" t="n"/>
     </row>
     <row r="8">
       <c r="D8" s="32" t="n"/>
-      <c r="E8" s="57" t="n"/>
-      <c r="F8" s="57" t="n"/>
-      <c r="G8" s="57" t="n"/>
-      <c r="H8" s="57" t="n"/>
-      <c r="I8" s="57" t="n"/>
-      <c r="J8" s="57" t="n"/>
-      <c r="K8" s="58" t="n"/>
     </row>
     <row r="9">
       <c r="D9" s="32" t="n"/>
-      <c r="E9" s="57" t="n"/>
-      <c r="F9" s="57" t="n"/>
-      <c r="G9" s="57" t="n"/>
-      <c r="H9" s="57" t="n"/>
-      <c r="I9" s="57" t="n"/>
-      <c r="J9" s="57" t="n"/>
-      <c r="K9" s="58" t="n"/>
     </row>
     <row r="10">
       <c r="D10" s="32" t="n"/>
-      <c r="E10" s="57" t="n"/>
-      <c r="F10" s="57" t="n"/>
-      <c r="G10" s="57" t="n"/>
-      <c r="H10" s="57" t="n"/>
-      <c r="I10" s="57" t="n"/>
-      <c r="J10" s="57" t="n"/>
-      <c r="K10" s="58" t="n"/>
     </row>
     <row r="11">
       <c r="D11" s="32" t="n"/>
-      <c r="E11" s="57" t="n"/>
-      <c r="F11" s="57" t="n"/>
-      <c r="G11" s="57" t="n"/>
-      <c r="H11" s="57" t="n"/>
-      <c r="I11" s="57" t="n"/>
-      <c r="J11" s="57" t="n"/>
-      <c r="K11" s="58" t="n"/>
     </row>
     <row r="12">
       <c r="D12" s="32" t="n"/>
-      <c r="E12" s="57" t="n"/>
-      <c r="F12" s="57" t="n"/>
-      <c r="G12" s="57" t="n"/>
-      <c r="H12" s="57" t="n"/>
-      <c r="I12" s="57" t="n"/>
-      <c r="J12" s="57" t="n"/>
-      <c r="K12" s="58" t="n"/>
     </row>
     <row r="13">
       <c r="D13" s="32" t="n"/>
-      <c r="E13" s="57" t="n"/>
-      <c r="F13" s="57" t="n"/>
-      <c r="G13" s="57" t="n"/>
-      <c r="H13" s="57" t="n"/>
-      <c r="I13" s="57" t="n"/>
-      <c r="J13" s="57" t="n"/>
-      <c r="K13" s="58" t="n"/>
     </row>
     <row r="14">
       <c r="D14" s="32" t="n"/>
-      <c r="E14" s="57" t="n"/>
-      <c r="F14" s="57" t="n"/>
-      <c r="G14" s="57" t="n"/>
-      <c r="H14" s="57" t="n"/>
-      <c r="I14" s="57" t="n"/>
-      <c r="J14" s="57" t="n"/>
-      <c r="K14" s="58" t="n"/>
     </row>
     <row r="15">
       <c r="D15" s="32" t="n"/>
-      <c r="E15" s="57" t="n"/>
-      <c r="F15" s="57" t="n"/>
-      <c r="G15" s="57" t="n"/>
-      <c r="H15" s="57" t="n"/>
-      <c r="I15" s="57" t="n"/>
-      <c r="J15" s="57" t="n"/>
-      <c r="K15" s="58" t="n"/>
     </row>
     <row r="16">
       <c r="D16" s="32" t="n"/>
-      <c r="E16" s="57" t="n"/>
-      <c r="F16" s="57" t="n"/>
-      <c r="G16" s="57" t="n"/>
-      <c r="H16" s="57" t="n"/>
-      <c r="I16" s="57" t="n"/>
-      <c r="J16" s="57" t="n"/>
-      <c r="K16" s="58" t="n"/>
-    </row>
+    </row>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
     <row r="31">
       <c r="D31" s="32" t="n"/>
-      <c r="E31" s="57" t="n"/>
-      <c r="F31" s="57" t="n"/>
-      <c r="G31" s="57" t="n"/>
-      <c r="H31" s="57" t="n"/>
-      <c r="I31" s="57" t="n"/>
-      <c r="J31" s="57" t="n"/>
-      <c r="K31" s="58" t="n"/>
     </row>
     <row r="32">
       <c r="D32" s="32" t="n"/>
-      <c r="E32" s="57" t="n"/>
-      <c r="F32" s="57" t="n"/>
-      <c r="G32" s="57" t="n"/>
-      <c r="H32" s="57" t="n"/>
-      <c r="I32" s="57" t="n"/>
-      <c r="J32" s="57" t="n"/>
-      <c r="K32" s="58" t="n"/>
     </row>
     <row r="33">
       <c r="D33" s="32" t="n"/>
-      <c r="E33" s="57" t="n"/>
-      <c r="F33" s="57" t="n"/>
-      <c r="G33" s="57" t="n"/>
-      <c r="H33" s="57" t="n"/>
-      <c r="I33" s="57" t="n"/>
-      <c r="J33" s="57" t="n"/>
-      <c r="K33" s="58" t="n"/>
     </row>
     <row r="34">
       <c r="D34" s="32" t="n"/>
-      <c r="E34" s="57" t="n"/>
-      <c r="F34" s="57" t="n"/>
-      <c r="G34" s="57" t="n"/>
-      <c r="H34" s="57" t="n"/>
-      <c r="I34" s="57" t="n"/>
-      <c r="J34" s="57" t="n"/>
-      <c r="K34" s="58" t="n"/>
     </row>
     <row r="35">
       <c r="D35" s="32" t="n"/>
-      <c r="E35" s="57" t="n"/>
-      <c r="F35" s="57" t="n"/>
-      <c r="G35" s="57" t="n"/>
-      <c r="H35" s="57" t="n"/>
-      <c r="I35" s="57" t="n"/>
-      <c r="J35" s="57" t="n"/>
-      <c r="K35" s="58" t="n"/>
     </row>
     <row r="36">
       <c r="D36" s="32" t="n"/>
-      <c r="E36" s="57" t="n"/>
-      <c r="F36" s="57" t="n"/>
-      <c r="G36" s="57" t="n"/>
-      <c r="H36" s="57" t="n"/>
-      <c r="I36" s="57" t="n"/>
-      <c r="J36" s="57" t="n"/>
-      <c r="K36" s="58" t="n"/>
     </row>
     <row r="37">
       <c r="D37" s="32" t="n"/>
-      <c r="E37" s="57" t="n"/>
-      <c r="F37" s="57" t="n"/>
-      <c r="G37" s="57" t="n"/>
-      <c r="H37" s="57" t="n"/>
-      <c r="I37" s="57" t="n"/>
-      <c r="J37" s="57" t="n"/>
-      <c r="K37" s="58" t="n"/>
     </row>
     <row r="38">
       <c r="D38" s="32" t="n"/>
-      <c r="E38" s="57" t="n"/>
-      <c r="F38" s="57" t="n"/>
-      <c r="G38" s="57" t="n"/>
-      <c r="H38" s="57" t="n"/>
-      <c r="I38" s="57" t="n"/>
-      <c r="J38" s="57" t="n"/>
-      <c r="K38" s="58" t="n"/>
     </row>
     <row r="39">
       <c r="D39" s="32" t="n"/>
-      <c r="E39" s="57" t="n"/>
-      <c r="F39" s="57" t="n"/>
-      <c r="G39" s="57" t="n"/>
-      <c r="H39" s="57" t="n"/>
-      <c r="I39" s="57" t="n"/>
-      <c r="J39" s="57" t="n"/>
-      <c r="K39" s="58" t="n"/>
     </row>
     <row r="40">
       <c r="D40" s="32" t="n"/>
-      <c r="E40" s="57" t="n"/>
-      <c r="F40" s="57" t="n"/>
-      <c r="G40" s="57" t="n"/>
-      <c r="H40" s="57" t="n"/>
-      <c r="I40" s="57" t="n"/>
-      <c r="J40" s="57" t="n"/>
-      <c r="K40" s="58" t="n"/>
     </row>
     <row r="41">
       <c r="D41" s="32" t="n"/>
-      <c r="E41" s="57" t="n"/>
-      <c r="F41" s="57" t="n"/>
-      <c r="G41" s="57" t="n"/>
-      <c r="H41" s="57" t="n"/>
-      <c r="I41" s="57" t="n"/>
-      <c r="J41" s="57" t="n"/>
-      <c r="K41" s="58" t="n"/>
     </row>
     <row r="42">
       <c r="D42" s="32" t="n"/>
-      <c r="E42" s="57" t="n"/>
-      <c r="F42" s="57" t="n"/>
-      <c r="G42" s="57" t="n"/>
-      <c r="H42" s="57" t="n"/>
-      <c r="I42" s="57" t="n"/>
-      <c r="J42" s="57" t="n"/>
-      <c r="K42" s="58" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="D34:K34"/>
-    <mergeCell ref="D10:K10"/>
-    <mergeCell ref="D31:K31"/>
-    <mergeCell ref="D40:K40"/>
-    <mergeCell ref="D36:K36"/>
-    <mergeCell ref="D6:K6"/>
-    <mergeCell ref="D11:K11"/>
-    <mergeCell ref="D13:K13"/>
-    <mergeCell ref="D41:K41"/>
-    <mergeCell ref="D32:K32"/>
-    <mergeCell ref="D7:K7"/>
-    <mergeCell ref="D16:K16"/>
-    <mergeCell ref="D37:K37"/>
-    <mergeCell ref="D4:K4"/>
-    <mergeCell ref="D12:K12"/>
-    <mergeCell ref="D9:K9"/>
-    <mergeCell ref="D39:K39"/>
-    <mergeCell ref="D8:K8"/>
-    <mergeCell ref="D15:K15"/>
-    <mergeCell ref="D33:K33"/>
-    <mergeCell ref="D42:K42"/>
-    <mergeCell ref="D38:K38"/>
-    <mergeCell ref="D14:K14"/>
-    <mergeCell ref="D5:K5"/>
-    <mergeCell ref="D35:K35"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" verticalDpi="0"/>
 </worksheet>
@@ -1894,7 +1744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:O114"/>
+  <dimension ref="A1:O114"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="16.5"/>
   <cols>
     <col width="2.625" customWidth="1" style="1" min="1" max="1"/>
@@ -1928,6 +1778,7 @@
       <c r="N2" s="18" t="n"/>
       <c r="O2" s="18" t="n"/>
     </row>
+    <row r="3" s="46"/>
     <row r="4" ht="17.25" customHeight="1" s="46">
       <c r="C4" s="16" t="inlineStr">
         <is>
@@ -1935,14 +1786,15 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" s="46">
       <c r="C5" s="14" t="inlineStr">
         <is>
           <t>- Provides convenience for quest location and direction</t>
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="6" s="46"/>
+    <row r="7" s="46">
       <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Display by Unit</t>
@@ -2254,84 +2106,84 @@
       <c r="M16" s="60" t="n"/>
       <c r="N16" s="59" t="n"/>
     </row>
-    <row r="17">
+    <row r="17" s="46">
       <c r="C17" s="14" t="n"/>
     </row>
-    <row r="18">
+    <row r="18" s="46">
       <c r="C18" s="15" t="inlineStr">
         <is>
           <t>Quest Navigation Guide</t>
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" s="46">
       <c r="C19" s="26" t="inlineStr">
         <is>
           <t>- Arrow indicators around the character guide the quest destination</t>
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" s="46">
       <c r="C20" s="14" t="n"/>
     </row>
-    <row r="21">
+    <row r="21" s="46">
       <c r="C21" s="14" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" s="46">
       <c r="C22" s="14" t="n"/>
     </row>
-    <row r="23">
+    <row r="23" s="46">
       <c r="C23" s="14" t="n"/>
     </row>
-    <row r="24">
+    <row r="24" s="46">
       <c r="C24" s="14" t="n"/>
     </row>
-    <row r="25">
+    <row r="25" s="46">
       <c r="C25" s="14" t="n"/>
     </row>
-    <row r="26">
+    <row r="26" s="46">
       <c r="C26" s="14" t="n"/>
     </row>
-    <row r="27">
+    <row r="27" s="46">
       <c r="C27" s="14" t="n"/>
     </row>
-    <row r="28">
+    <row r="28" s="46">
       <c r="C28" s="14" t="n"/>
     </row>
-    <row r="29">
+    <row r="29" s="46">
       <c r="C29" s="14" t="n"/>
     </row>
-    <row r="30">
+    <row r="30" s="46">
       <c r="C30" s="14" t="n"/>
     </row>
-    <row r="31">
+    <row r="31" s="46">
       <c r="C31" s="14" t="n"/>
     </row>
-    <row r="32">
+    <row r="32" s="46">
       <c r="C32" s="14" t="n"/>
     </row>
-    <row r="33">
+    <row r="33" s="46">
       <c r="C33" s="14" t="n"/>
     </row>
-    <row r="34">
+    <row r="34" s="46">
       <c r="C34" s="14" t="n"/>
     </row>
-    <row r="35">
+    <row r="35" s="46">
       <c r="C35" s="14" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" s="46">
       <c r="C36" s="14" t="n"/>
     </row>
-    <row r="37">
+    <row r="37" s="46">
       <c r="C37" s="14" t="n"/>
     </row>
-    <row r="38">
+    <row r="38" s="46">
       <c r="C38" s="14" t="n"/>
     </row>
-    <row r="39">
+    <row r="39" s="46">
       <c r="C39" s="14" t="n"/>
     </row>
-    <row r="40">
+    <row r="40" s="46">
       <c r="C40" s="14" t="n"/>
     </row>
     <row r="41" ht="17.25" customHeight="1" s="46">
@@ -2381,11 +2233,7 @@
       </c>
       <c r="D43" s="42" t="inlineStr">
         <is>
-          <t>Quest Guide effect displayed arrow displayed. arrow periodically 
-- move possible ‘’ 
-defeat , Quest Monster placement zone PC displayed 
-gimmick gimmick placement zone PC displayed 
-- cutscene displayed</t>
+          <t>Quest Guide effect displayed arrow displayed. arrow periodically - move possible ‘’ defeat , Quest Monster placement zone PC displayed gimmick placement zone PC displayed - cutscene displayed</t>
         </is>
       </c>
       <c r="E43" s="60" t="n"/>
@@ -2396,90 +2244,90 @@
       <c r="J43" s="60" t="n"/>
       <c r="K43" s="59" t="n"/>
     </row>
-    <row r="44">
+    <row r="44" s="46">
       <c r="C44" s="14" t="n"/>
     </row>
-    <row r="45">
+    <row r="45" s="46">
       <c r="C45" s="15" t="inlineStr">
         <is>
           <t>Guide Effect</t>
         </is>
       </c>
     </row>
-    <row r="46">
+    <row r="46" s="46">
       <c r="C46" s="26" t="inlineStr">
         <is>
           <t>- Effect directly marking the quest objective</t>
         </is>
       </c>
     </row>
-    <row r="47">
+    <row r="47" s="46">
       <c r="C47" s="14" t="n"/>
     </row>
-    <row r="48">
+    <row r="48" s="46">
       <c r="C48" s="14" t="n"/>
     </row>
-    <row r="49">
+    <row r="49" s="46">
       <c r="C49" s="14" t="n"/>
     </row>
-    <row r="50">
+    <row r="50" s="46">
       <c r="C50" s="14" t="n"/>
     </row>
-    <row r="51">
+    <row r="51" s="46">
       <c r="C51" s="14" t="n"/>
     </row>
-    <row r="52">
+    <row r="52" s="46">
       <c r="C52" s="14" t="n"/>
     </row>
-    <row r="53">
+    <row r="53" s="46">
       <c r="C53" s="14" t="n"/>
     </row>
-    <row r="54">
+    <row r="54" s="46">
       <c r="C54" s="14" t="n"/>
     </row>
-    <row r="55">
+    <row r="55" s="46">
       <c r="C55" s="14" t="n"/>
     </row>
-    <row r="56">
+    <row r="56" s="46">
       <c r="C56" s="14" t="n"/>
     </row>
-    <row r="57">
+    <row r="57" s="46">
       <c r="C57" s="14" t="n"/>
     </row>
-    <row r="58">
+    <row r="58" s="46">
       <c r="C58" s="14" t="n"/>
     </row>
-    <row r="59">
+    <row r="59" s="46">
       <c r="C59" s="14" t="n"/>
     </row>
-    <row r="60">
+    <row r="60" s="46">
       <c r="C60" s="14" t="n"/>
     </row>
-    <row r="61">
+    <row r="61" s="46">
       <c r="C61" s="14" t="n"/>
     </row>
-    <row r="62">
+    <row r="62" s="46">
       <c r="C62" s="14" t="n"/>
     </row>
-    <row r="63">
+    <row r="63" s="46">
       <c r="C63" s="14" t="n"/>
     </row>
-    <row r="64">
+    <row r="64" s="46">
       <c r="C64" s="14" t="n"/>
     </row>
-    <row r="65">
+    <row r="65" s="46">
       <c r="C65" s="14" t="n"/>
     </row>
-    <row r="66">
+    <row r="66" s="46">
       <c r="C66" s="14" t="n"/>
     </row>
-    <row r="67">
+    <row r="67" s="46">
       <c r="C67" s="14" t="n"/>
     </row>
-    <row r="68">
+    <row r="68" s="46">
       <c r="C68" s="14" t="n"/>
     </row>
-    <row r="69">
+    <row r="69" s="46">
       <c r="C69" s="23" t="inlineStr">
         <is>
           <t>time(s)</t>
@@ -2582,49 +2430,77 @@
       <c r="M72" s="60" t="n"/>
       <c r="N72" s="59" t="n"/>
     </row>
-    <row r="73">
+    <row r="73" s="46">
       <c r="C73" s="14" t="n"/>
     </row>
-    <row r="74">
+    <row r="74" s="46">
       <c r="C74" s="15" t="inlineStr">
         <is>
           <t>Quest Monster Guide</t>
         </is>
       </c>
     </row>
-    <row r="75">
+    <row r="75" s="46">
       <c r="C75" s="25" t="inlineStr">
         <is>
           <t>- Exclamation mark displayed above monster's head</t>
         </is>
       </c>
     </row>
-    <row r="76">
+    <row r="76" s="46">
       <c r="C76" s="14" t="n"/>
     </row>
-    <row r="77">
+    <row r="77" s="46">
       <c r="C77" s="14" t="n"/>
     </row>
-    <row r="78">
+    <row r="78" s="46">
       <c r="C78" s="14" t="n"/>
     </row>
-    <row r="79">
+    <row r="79" s="46">
       <c r="C79" s="14" t="n"/>
     </row>
-    <row r="80">
+    <row r="80" s="46">
       <c r="C80" s="14" t="n"/>
     </row>
-    <row r="81">
+    <row r="81" s="46">
       <c r="C81" s="14" t="n"/>
     </row>
-    <row r="93">
+    <row r="82" s="46"/>
+    <row r="83" s="46"/>
+    <row r="84" s="46"/>
+    <row r="85" s="46"/>
+    <row r="86" s="46"/>
+    <row r="87" s="46"/>
+    <row r="88" s="46"/>
+    <row r="89" s="46"/>
+    <row r="90" s="46"/>
+    <row r="91" s="46"/>
+    <row r="92" s="46"/>
+    <row r="93" s="46">
       <c r="C93" s="15" t="inlineStr">
         <is>
           <t>Minimap Marking</t>
         </is>
       </c>
     </row>
-    <row r="111">
+    <row r="94" s="46"/>
+    <row r="95" s="46"/>
+    <row r="96" s="46"/>
+    <row r="97" s="46"/>
+    <row r="98" s="46"/>
+    <row r="99" s="46"/>
+    <row r="100" s="46"/>
+    <row r="101" s="46"/>
+    <row r="102" s="46"/>
+    <row r="103" s="46"/>
+    <row r="104" s="46"/>
+    <row r="105" s="46"/>
+    <row r="106" s="46"/>
+    <row r="107" s="46"/>
+    <row r="108" s="46"/>
+    <row r="109" s="46"/>
+    <row r="110" s="46"/>
+    <row r="111" s="46">
       <c r="C111" s="23" t="inlineStr">
         <is>
           <t>time(s)</t>

</xml_diff>

<commit_message>
Add IP protection: CONFIDENTIAL watermarks, data masking, image redaction
- All 43 sheets across 7 XLSX files: CONFIDENTIAL header added
- 2,284 balance/reward data cells masked in SeasonPass, Exploration, Records
- 358 design images blurred + CONFIDENTIAL watermark overlay
- Protects unreleased game IP while maintaining portfolio structure
</commit_message>
<xml_diff>
--- a/docs/QuestGuide_DesignDocument.xlsx
+++ b/docs/QuestGuide_DesignDocument.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="맑은 고딕"/>
       <charset val="129"/>
@@ -139,8 +139,15 @@
       <name val="맑은 고딕"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00CC0000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -159,6 +166,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2F2"/>
+        <bgColor rgb="00FFF2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="43">
     <border>
@@ -692,7 +705,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -876,6 +889,9 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1541,124 +1557,128 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L42"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="4.375" customWidth="1" style="32" min="1" max="1"/>
     <col width="8" customWidth="1" style="32" min="2" max="2"/>
     <col width="12" customWidth="1" style="32" min="3" max="3"/>
     <col width="75" customWidth="1" style="32" min="4" max="15"/>
-    <col width="18" customWidth="1" style="46" min="5" max="5"/>
-    <col width="8.43" customWidth="1" style="46" min="12" max="12"/>
+    <col width="18" customWidth="1" style="46" min="12" max="12"/>
     <col width="11.375" bestFit="1" customWidth="1" style="32" min="16" max="16"/>
     <col width="9" customWidth="1" style="32" min="17" max="16384"/>
   </cols>
   <sheetData>
-    <row r="2" ht="22" customHeight="1" s="46">
-      <c r="B2" s="61" t="inlineStr">
+    <row r="1" ht="25" customHeight="1" s="46">
+      <c r="A1" s="70" t="inlineStr">
+        <is>
+          <t>CONFIDENTIAL — Shared for portfolio review purposes only. All game content is the property of its respective studio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1" s="46"/>
+    <row r="3" ht="18" customHeight="1" s="46">
+      <c r="B3" s="61" t="inlineStr">
         <is>
           <t>Document History : Quest Guide System</t>
         </is>
       </c>
-      <c r="C2" s="5" t="n"/>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="5" t="n"/>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="5" t="n"/>
-      <c r="J2" s="5" t="n"/>
-      <c r="K2" s="5" t="n"/>
-      <c r="L2" s="5" t="n"/>
-    </row>
-    <row r="3" ht="18" customHeight="1" s="46">
-      <c r="B3" s="62" t="inlineStr">
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="5" t="n"/>
+      <c r="K3" s="5" t="n"/>
+      <c r="L3" s="5" t="n"/>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="46">
+      <c r="B4" s="62" t="inlineStr">
         <is>
           <t>Index</t>
         </is>
       </c>
-      <c r="C3" s="62" t="inlineStr">
+      <c r="C4" s="62" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="D3" s="62" t="inlineStr">
+      <c r="D4" s="62" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Author</t>
         </is>
       </c>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
-      <c r="J3" s="6" t="n"/>
-      <c r="K3" s="6" t="n"/>
-      <c r="L3" s="62" t="n"/>
-    </row>
-    <row r="4" ht="18" customHeight="1" s="46">
-      <c r="A4" s="7" t="n"/>
-      <c r="B4" s="63" t="n">
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="n"/>
+      <c r="K4" s="6" t="n"/>
+      <c r="L4" s="62" t="n"/>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="46">
+      <c r="A5" s="7" t="n"/>
+      <c r="B5" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="64" t="inlineStr">
+      <c r="C5" s="64" t="inlineStr">
         <is>
           <t>24.05.03</t>
         </is>
       </c>
-      <c r="D4" s="64" t="inlineStr">
+      <c r="D5" s="64" t="inlineStr">
         <is>
           <t>Initial draft</t>
         </is>
       </c>
-      <c r="E4" s="0" t="inlineStr">
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
-      <c r="L4" s="65" t="n"/>
-    </row>
-    <row r="5" ht="18" customHeight="1" s="46">
-      <c r="A5" s="30" t="n"/>
-      <c r="B5" s="66" t="n">
-        <v>2</v>
-      </c>
-      <c r="C5" s="67" t="inlineStr">
-        <is>
-          <t>25.06.11</t>
-        </is>
-      </c>
-      <c r="D5" s="68" t="inlineStr">
-        <is>
-          <t>UI updated; detailed descriptions added</t>
-        </is>
-      </c>
-      <c r="E5" s="0" t="inlineStr">
-        <is>
-          <t>Juwon Lee</t>
-        </is>
-      </c>
-      <c r="L5" s="69" t="n"/>
+      <c r="L5" s="65" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="30" t="n"/>
-      <c r="B6" s="31" t="n"/>
-      <c r="C6" s="28" t="n"/>
-      <c r="D6" s="52" t="n"/>
-      <c r="L6" s="27" t="n"/>
+      <c r="B6" s="66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="67" t="inlineStr">
+        <is>
+          <t>25.06.11</t>
+        </is>
+      </c>
+      <c r="D6" s="68" t="inlineStr">
+        <is>
+          <t>UI updated; detailed descriptions added</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>Juwon Lee</t>
+        </is>
+      </c>
+      <c r="L6" s="69" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="40" t="n"/>
-      <c r="C7" s="40" t="n"/>
-      <c r="D7" s="40" t="n"/>
-      <c r="L7" s="40" t="n"/>
+      <c r="A7" s="30" t="n"/>
+      <c r="B7" s="31" t="n"/>
+      <c r="C7" s="28" t="n"/>
+      <c r="D7" s="52" t="n"/>
+      <c r="L7" s="27" t="n"/>
     </row>
     <row r="8">
-      <c r="D8" s="32" t="n"/>
+      <c r="B8" s="40" t="n"/>
+      <c r="C8" s="40" t="n"/>
+      <c r="D8" s="40" t="n"/>
+      <c r="L8" s="40" t="n"/>
     </row>
     <row r="9">
       <c r="D9" s="32" t="n"/>
@@ -1684,8 +1704,8 @@
     <row r="16">
       <c r="D16" s="32" t="n"/>
     </row>
-    <row r="31">
-      <c r="D31" s="32" t="n"/>
+    <row r="17">
+      <c r="D17" s="32" t="n"/>
     </row>
     <row r="32">
       <c r="D32" s="32" t="n"/>
@@ -1720,7 +1740,13 @@
     <row r="42">
       <c r="D42" s="32" t="n"/>
     </row>
+    <row r="43">
+      <c r="D43" s="32" t="n"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" verticalDpi="0"/>
 </worksheet>
@@ -1732,7 +1758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:O114"/>
+  <dimension ref="A1:O115"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="16.5"/>
   <cols>
     <col width="2.625" customWidth="1" style="1" min="1" max="1"/>
@@ -1745,118 +1771,88 @@
     <col width="8.625" customWidth="1" style="1" min="9" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="3.95" customHeight="1" s="46"/>
-    <row r="2" ht="27.95" customHeight="1" s="46">
-      <c r="B2" s="18" t="inlineStr">
+    <row r="1" ht="25" customHeight="1" s="46">
+      <c r="A1" s="70" t="inlineStr">
+        <is>
+          <t>CONFIDENTIAL — Shared for portfolio review purposes only. All game content is the property of its respective studio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="27.95" customHeight="1" s="46"/>
+    <row r="3" s="46">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>Quest Guide System</t>
         </is>
       </c>
-      <c r="C2" s="18" t="n"/>
-      <c r="D2" s="18" t="n"/>
-      <c r="E2" s="18" t="n"/>
-      <c r="F2" s="18" t="n"/>
-      <c r="G2" s="18" t="n"/>
-      <c r="H2" s="18" t="n"/>
-      <c r="I2" s="18" t="n"/>
-      <c r="J2" s="18" t="n"/>
-      <c r="K2" s="18" t="n"/>
-      <c r="L2" s="18" t="n"/>
-      <c r="M2" s="18" t="n"/>
-      <c r="N2" s="18" t="n"/>
-      <c r="O2" s="18" t="n"/>
-    </row>
-    <row r="3" s="46"/>
-    <row r="4" ht="17.25" customHeight="1" s="46">
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C3" s="18" t="n"/>
+      <c r="D3" s="18" t="n"/>
+      <c r="E3" s="18" t="n"/>
+      <c r="F3" s="18" t="n"/>
+      <c r="G3" s="18" t="n"/>
+      <c r="H3" s="18" t="n"/>
+      <c r="I3" s="18" t="n"/>
+      <c r="J3" s="18" t="n"/>
+      <c r="K3" s="18" t="n"/>
+      <c r="L3" s="18" t="n"/>
+      <c r="M3" s="18" t="n"/>
+      <c r="N3" s="18" t="n"/>
+      <c r="O3" s="18" t="n"/>
+    </row>
+    <row r="4" ht="17.25" customHeight="1" s="46"/>
+    <row r="5" s="46">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>Design Intent</t>
         </is>
       </c>
     </row>
-    <row r="5" s="46">
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>- Provides navigational convenience for quest locations and directions</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" s="46"/>
-    <row r="7" s="46">
-      <c r="C7" s="15" t="inlineStr">
+    <row r="6" s="46">
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>- Provides convenience for quest location and direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" s="46"/>
+    <row r="8" ht="35.25" customHeight="1" s="46">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>Display by Unit</t>
         </is>
       </c>
-      <c r="D7" s="20" t="n"/>
-      <c r="E7" s="21" t="n"/>
-      <c r="F7" s="20" t="n"/>
-      <c r="G7" s="20" t="n"/>
-      <c r="H7" s="20" t="n"/>
-      <c r="I7" s="21" t="n"/>
-      <c r="J7" s="21" t="n"/>
-      <c r="K7" s="21" t="n"/>
-      <c r="L7" s="21" t="n"/>
-      <c r="M7" s="21" t="n"/>
-      <c r="N7" s="21" t="n"/>
-    </row>
-    <row r="8" ht="35.25" customHeight="1" s="46">
-      <c r="C8" s="41" t="inlineStr">
+      <c r="E8" s="21" t="n"/>
+      <c r="F8" s="20" t="n"/>
+      <c r="G8" s="20" t="n"/>
+      <c r="H8" s="20" t="n"/>
+    </row>
+    <row r="9" ht="31.5" customHeight="1" s="46">
+      <c r="C9" s="41" t="inlineStr">
         <is>
           <t>Quest Condition</t>
         </is>
       </c>
-      <c r="D8" s="59" t="n"/>
-      <c r="E8" s="41" t="inlineStr">
+      <c r="D9" s="59" t="n"/>
+      <c r="E9" s="41" t="inlineStr">
         <is>
           <t>Navigation Guide</t>
         </is>
       </c>
-      <c r="F8" s="41" t="inlineStr">
+      <c r="F9" s="41" t="inlineStr">
         <is>
           <t>Guide Effect</t>
         </is>
       </c>
-      <c r="G8" s="41" t="inlineStr">
-        <is>
-          <t>Minimap</t>
-        </is>
-      </c>
-      <c r="H8" s="41" t="inlineStr">
+      <c r="G9" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="H9" s="41" t="inlineStr">
         <is>
           <t>Special Notes</t>
         </is>
       </c>
-      <c r="I8" s="60" t="n"/>
-      <c r="J8" s="60" t="n"/>
-      <c r="K8" s="60" t="n"/>
-      <c r="L8" s="60" t="n"/>
-      <c r="M8" s="60" t="n"/>
-      <c r="N8" s="59" t="n"/>
-    </row>
-    <row r="9" ht="31.5" customHeight="1" s="46">
-      <c r="C9" s="43" t="inlineStr">
-        <is>
-          <t>CondTutorial</t>
-        </is>
-      </c>
-      <c r="D9" s="59" t="n"/>
-      <c r="E9" s="43" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F9" s="43" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G9" s="43" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H9" s="43" t="n"/>
       <c r="I9" s="60" t="n"/>
       <c r="J9" s="60" t="n"/>
       <c r="K9" s="60" t="n"/>
@@ -1867,23 +1863,23 @@
     <row r="10" ht="31.5" customHeight="1" s="46">
       <c r="C10" s="43" t="inlineStr">
         <is>
-          <t>CondDialog</t>
+          <t>CondTutorial</t>
         </is>
       </c>
       <c r="D10" s="59" t="n"/>
       <c r="E10" s="43" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="F10" s="43" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="G10" s="43" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="H10" s="43" t="n"/>
@@ -1897,7 +1893,7 @@
     <row r="11" ht="34.5" customHeight="1" s="46">
       <c r="C11" s="43" t="inlineStr">
         <is>
-          <t>CondMonster</t>
+          <t>CondDialog</t>
         </is>
       </c>
       <c r="D11" s="59" t="n"/>
@@ -1916,12 +1912,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="H11" s="43" t="inlineStr">
-        <is>
-          <t>• Guide effect displayed above the target monster
-• Navigation guide shown only in regions where the quest monster is not present</t>
-        </is>
-      </c>
+      <c r="H11" s="43" t="n"/>
       <c r="I11" s="60" t="n"/>
       <c r="J11" s="60" t="n"/>
       <c r="K11" s="60" t="n"/>
@@ -1932,7 +1923,7 @@
     <row r="12" ht="44.25" customHeight="1" s="46">
       <c r="C12" s="43" t="inlineStr">
         <is>
-          <t>CondItem</t>
+          <t>CondMonster</t>
         </is>
       </c>
       <c r="D12" s="59" t="n"/>
@@ -1953,8 +1944,8 @@
       </c>
       <c r="H12" s="43" t="inlineStr">
         <is>
-          <t>• Guide effect displayed above monsters that drop the target item
-• Navigation guide shown only in regions where item-dropping monsters are not present</t>
+          <t>• Guide effect displayed above target monster's head
+• Navigation guide displayed only in areas where the quest monster is not placed</t>
         </is>
       </c>
       <c r="I12" s="60" t="n"/>
@@ -1967,7 +1958,7 @@
     <row r="13" ht="24" customHeight="1" s="46">
       <c r="C13" s="43" t="inlineStr">
         <is>
-          <t>CondCutscene</t>
+          <t>CondItem</t>
         </is>
       </c>
       <c r="D13" s="59" t="n"/>
@@ -1986,7 +1977,12 @@
           <t>O</t>
         </is>
       </c>
-      <c r="H13" s="43" t="n"/>
+      <c r="H13" s="43" t="inlineStr">
+        <is>
+          <t>• Guide effect displayed above monsters that drop target items
+• Navigation guide displayed only in areas where item-dropping monsters are not placed</t>
+        </is>
+      </c>
       <c r="I13" s="60" t="n"/>
       <c r="J13" s="60" t="n"/>
       <c r="K13" s="60" t="n"/>
@@ -1997,7 +1993,7 @@
     <row r="14" ht="21.75" customHeight="1" s="46">
       <c r="C14" s="43" t="inlineStr">
         <is>
-          <t>CondArea</t>
+          <t>CondCutscene</t>
         </is>
       </c>
       <c r="D14" s="59" t="n"/>
@@ -2027,7 +2023,7 @@
     <row r="15" ht="46.5" customHeight="1" s="46">
       <c r="C15" s="43" t="inlineStr">
         <is>
-          <t>CondGimmick</t>
+          <t>CondArea</t>
         </is>
       </c>
       <c r="D15" s="59" t="n"/>
@@ -2046,13 +2042,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="H15" s="43" t="inlineStr">
-        <is>
-          <t>• When multiple quest gimmicks are targets:
-  ◦ Guide effect displayed for all gimmicks
-  ◦ Navigation guide shown only in regions where the gimmick is absent</t>
-        </is>
-      </c>
+      <c r="H15" s="43" t="n"/>
       <c r="I15" s="60" t="n"/>
       <c r="J15" s="60" t="n"/>
       <c r="K15" s="60" t="n"/>
@@ -2063,7 +2053,7 @@
     <row r="16" ht="21.75" customHeight="1" s="46">
       <c r="C16" s="43" t="inlineStr">
         <is>
-          <t>CondIndun</t>
+          <t>CondGimmick</t>
         </is>
       </c>
       <c r="D16" s="59" t="n"/>
@@ -2084,7 +2074,9 @@
       </c>
       <c r="H16" s="43" t="inlineStr">
         <is>
-          <t>• The gimmick granting entry to the Instanced Dungeon is marked as the target</t>
+          <t>• When multiple quest gimmicks are targets
+    ◦ Guide effect displayed for all gimmicks
+    ◦ Navigation guide displayed only in areas without those gimmicks</t>
         </is>
       </c>
       <c r="I16" s="60" t="n"/>
@@ -2095,24 +2087,55 @@
       <c r="N16" s="59" t="n"/>
     </row>
     <row r="17" s="46">
-      <c r="C17" s="14" t="n"/>
+      <c r="C17" s="43" t="inlineStr">
+        <is>
+          <t>CondIndun</t>
+        </is>
+      </c>
+      <c r="D17" s="59" t="n"/>
+      <c r="E17" s="43" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F17" s="43" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="G17" s="43" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="H17" s="43" t="inlineStr">
+        <is>
+          <t>• Gimmick allowing entry to the Instance Dungeon marked as target</t>
+        </is>
+      </c>
+      <c r="I17" s="60" t="n"/>
+      <c r="J17" s="60" t="n"/>
+      <c r="K17" s="60" t="n"/>
+      <c r="L17" s="60" t="n"/>
+      <c r="M17" s="60" t="n"/>
+      <c r="N17" s="59" t="n"/>
     </row>
     <row r="18" s="46">
-      <c r="C18" s="15" t="inlineStr">
+      <c r="C18" s="14" t="n"/>
+    </row>
+    <row r="19" s="46">
+      <c r="C19" s="15" t="inlineStr">
         <is>
           <t>Quest Navigation Guide</t>
         </is>
       </c>
     </row>
-    <row r="19" s="46">
-      <c r="C19" s="26" t="inlineStr">
+    <row r="20" s="46">
+      <c r="C20" s="26" t="inlineStr">
         <is>
           <t>- Arrow indicators around the character guide the quest destination</t>
         </is>
       </c>
-    </row>
-    <row r="20" s="46">
-      <c r="C20" s="14" t="n"/>
     </row>
     <row r="21" s="46">
       <c r="C21" s="14" t="n"/>
@@ -2175,36 +2198,17 @@
       <c r="C40" s="14" t="n"/>
     </row>
     <row r="41" ht="17.25" customHeight="1" s="46">
-      <c r="C41" s="17" t="inlineStr">
+      <c r="C41" s="14" t="n"/>
+    </row>
+    <row r="42" ht="84.75" customHeight="1" s="46">
+      <c r="C42" s="17" t="inlineStr">
         <is>
           <t>time(s)</t>
         </is>
       </c>
-      <c r="D41" s="45" t="inlineStr">
+      <c r="D42" s="45" t="inlineStr">
         <is>
           <t>Description</t>
-        </is>
-      </c>
-      <c r="E41" s="60" t="n"/>
-      <c r="F41" s="60" t="n"/>
-      <c r="G41" s="60" t="n"/>
-      <c r="H41" s="60" t="n"/>
-      <c r="I41" s="60" t="n"/>
-      <c r="J41" s="60" t="n"/>
-      <c r="K41" s="59" t="n"/>
-    </row>
-    <row r="42" ht="84.75" customHeight="1" s="46">
-      <c r="C42" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="42" t="inlineStr">
-        <is>
-          <t>My Display On/Off Button
-- Click when, Quest Guide Direction Display, Not Display before
- → Display during state in Click when, Not Display
- → Not Display during state in Click when, Display
-- Display state in Corresponding Icon Color to Display
-- Not Display state in Corresponding Icon Greyscale processing</t>
         </is>
       </c>
       <c r="E42" s="60" t="n"/>
@@ -2217,11 +2221,16 @@
     </row>
     <row r="43" ht="62.25" customHeight="1" s="46">
       <c r="C43" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D43" s="42" t="inlineStr">
         <is>
-          <t>Quest Guide effect displayed arrow displayed. arrow periodically - move possible ‘’ defeat , Quest Monster placement zone PC displayed gimmick placement zone PC displayed - cutscene displayed</t>
+          <t>My Display On/Off Button
+- Click when, Quest Guide Direction Display, Not Display before
+ → Display during state in Click when, Not Display
+ → Not Display during state in Click when, Display
+- Display state in Corresponding Icon Color to Display
+- Not Display state in Corresponding Icon Greyscale processing</t>
         </is>
       </c>
       <c r="E43" s="60" t="n"/>
@@ -2233,24 +2242,38 @@
       <c r="K43" s="59" t="n"/>
     </row>
     <row r="44" s="46">
-      <c r="C44" s="14" t="n"/>
+      <c r="C44" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" s="42" t="inlineStr">
+        <is>
+          <t>Quest Guide effect displayed arrow displayed. arrow periodically - move possible ‘’ defeat , Quest Monster placement zone PC displayed gimmick placement zone PC displayed - cutscene displayed</t>
+        </is>
+      </c>
+      <c r="E44" s="60" t="n"/>
+      <c r="F44" s="60" t="n"/>
+      <c r="G44" s="60" t="n"/>
+      <c r="H44" s="60" t="n"/>
+      <c r="I44" s="60" t="n"/>
+      <c r="J44" s="60" t="n"/>
+      <c r="K44" s="59" t="n"/>
     </row>
     <row r="45" s="46">
-      <c r="C45" s="15" t="inlineStr">
+      <c r="C45" s="14" t="n"/>
+    </row>
+    <row r="46" s="46">
+      <c r="C46" s="15" t="inlineStr">
         <is>
           <t>Guide Effect</t>
         </is>
       </c>
     </row>
-    <row r="46" s="46">
-      <c r="C46" s="26" t="inlineStr">
+    <row r="47" s="46">
+      <c r="C47" s="26" t="inlineStr">
         <is>
           <t>- Effect directly marking the quest objective</t>
         </is>
       </c>
-    </row>
-    <row r="47" s="46">
-      <c r="C47" s="14" t="n"/>
     </row>
     <row r="48" s="46">
       <c r="C48" s="14" t="n"/>
@@ -2316,34 +2339,17 @@
       <c r="C68" s="14" t="n"/>
     </row>
     <row r="69" s="46">
-      <c r="C69" s="23" t="inlineStr">
+      <c r="C69" s="14" t="n"/>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="46">
+      <c r="C70" s="23" t="inlineStr">
         <is>
           <t>time(s)</t>
         </is>
       </c>
-      <c r="D69" s="42" t="inlineStr">
+      <c r="D70" s="42" t="inlineStr">
         <is>
           <t>Description</t>
-        </is>
-      </c>
-      <c r="E69" s="60" t="n"/>
-      <c r="F69" s="60" t="n"/>
-      <c r="G69" s="60" t="n"/>
-      <c r="H69" s="60" t="n"/>
-      <c r="I69" s="60" t="n"/>
-      <c r="J69" s="60" t="n"/>
-      <c r="K69" s="60" t="n"/>
-      <c r="L69" s="60" t="n"/>
-      <c r="M69" s="60" t="n"/>
-      <c r="N69" s="59" t="n"/>
-    </row>
-    <row r="70" ht="16.5" customHeight="1" s="46">
-      <c r="C70" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="D70" s="42" t="inlineStr">
-        <is>
-          <t>Location guide for specific points, NPCs, gimmick objects</t>
         </is>
       </c>
       <c r="E70" s="60" t="n"/>
@@ -2358,12 +2364,32 @@
       <c r="N70" s="59" t="n"/>
     </row>
     <row r="71" ht="210.75" customHeight="1" s="46">
-      <c r="C71" s="24" t="inlineStr">
+      <c r="C71" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" s="42" t="inlineStr">
+        <is>
+          <t>Location guide for specific points, NPCs, gimmick objects</t>
+        </is>
+      </c>
+      <c r="E71" s="60" t="n"/>
+      <c r="F71" s="60" t="n"/>
+      <c r="G71" s="60" t="n"/>
+      <c r="H71" s="60" t="n"/>
+      <c r="I71" s="60" t="n"/>
+      <c r="J71" s="60" t="n"/>
+      <c r="K71" s="60" t="n"/>
+      <c r="L71" s="60" t="n"/>
+      <c r="M71" s="60" t="n"/>
+      <c r="N71" s="59" t="n"/>
+    </row>
+    <row r="72" ht="46.5" customHeight="1" s="46">
+      <c r="C72" s="24" t="inlineStr">
         <is>
           <t>Display Conditions</t>
         </is>
       </c>
-      <c r="D71" s="42" t="inlineStr">
+      <c r="D72" s="42" t="inlineStr">
         <is>
           <t>in progress 
 - QuestMissionList status list
@@ -2383,30 +2409,6 @@
 - cutscene displayed</t>
         </is>
       </c>
-      <c r="E71" s="60" t="n"/>
-      <c r="F71" s="60" t="n"/>
-      <c r="G71" s="60" t="n"/>
-      <c r="H71" s="60" t="n"/>
-      <c r="I71" s="60" t="n"/>
-      <c r="J71" s="60" t="n"/>
-      <c r="K71" s="60" t="n"/>
-      <c r="L71" s="60" t="n"/>
-      <c r="M71" s="60" t="n"/>
-      <c r="N71" s="59" t="n"/>
-    </row>
-    <row r="72" ht="46.5" customHeight="1" s="46">
-      <c r="C72" s="24" t="inlineStr">
-        <is>
-          <t>Quest Effect</t>
-        </is>
-      </c>
-      <c r="D72" s="42" t="inlineStr">
-        <is>
-          <t>- Effect names
-    ◦ QuestCompleteLoop01
-    ◦ QuestCompleteShot01</t>
-        </is>
-      </c>
       <c r="E72" s="60" t="n"/>
       <c r="F72" s="60" t="n"/>
       <c r="G72" s="60" t="n"/>
@@ -2419,24 +2421,45 @@
       <c r="N72" s="59" t="n"/>
     </row>
     <row r="73" s="46">
-      <c r="C73" s="14" t="n"/>
+      <c r="C73" s="24" t="inlineStr">
+        <is>
+          <t>Quest Effect</t>
+        </is>
+      </c>
+      <c r="D73" s="42" t="inlineStr">
+        <is>
+          <t>- Effect names
+    ◦ QuestCompleteLoop01
+    ◦ QuestCompleteShot01</t>
+        </is>
+      </c>
+      <c r="E73" s="60" t="n"/>
+      <c r="F73" s="60" t="n"/>
+      <c r="G73" s="60" t="n"/>
+      <c r="H73" s="60" t="n"/>
+      <c r="I73" s="60" t="n"/>
+      <c r="J73" s="60" t="n"/>
+      <c r="K73" s="60" t="n"/>
+      <c r="L73" s="60" t="n"/>
+      <c r="M73" s="60" t="n"/>
+      <c r="N73" s="59" t="n"/>
     </row>
     <row r="74" s="46">
-      <c r="C74" s="15" t="inlineStr">
+      <c r="C74" s="14" t="n"/>
+    </row>
+    <row r="75" s="46">
+      <c r="C75" s="15" t="inlineStr">
         <is>
           <t>Quest Monster Guide</t>
         </is>
       </c>
     </row>
-    <row r="75" s="46">
-      <c r="C75" s="25" t="inlineStr">
+    <row r="76" s="46">
+      <c r="C76" s="25" t="inlineStr">
         <is>
           <t>- Exclamation mark displayed above monster's head</t>
         </is>
       </c>
-    </row>
-    <row r="76" s="46">
-      <c r="C76" s="14" t="n"/>
     </row>
     <row r="77" s="46">
       <c r="C77" s="14" t="n"/>
@@ -2453,7 +2476,9 @@
     <row r="81" s="46">
       <c r="C81" s="14" t="n"/>
     </row>
-    <row r="82" s="46"/>
+    <row r="82" s="46">
+      <c r="C82" s="14" t="n"/>
+    </row>
     <row r="83" s="46"/>
     <row r="84" s="46"/>
     <row r="85" s="46"/>
@@ -2464,14 +2489,14 @@
     <row r="90" s="46"/>
     <row r="91" s="46"/>
     <row r="92" s="46"/>
-    <row r="93" s="46">
-      <c r="C93" s="15" t="inlineStr">
+    <row r="93" s="46"/>
+    <row r="94" s="46">
+      <c r="C94" s="15" t="inlineStr">
         <is>
           <t>Minimap Marking</t>
         </is>
       </c>
     </row>
-    <row r="94" s="46"/>
     <row r="95" s="46"/>
     <row r="96" s="46"/>
     <row r="97" s="46"/>
@@ -2488,37 +2513,16 @@
     <row r="108" s="46"/>
     <row r="109" s="46"/>
     <row r="110" s="46"/>
-    <row r="111" s="46">
-      <c r="C111" s="23" t="inlineStr">
+    <row r="111" s="46"/>
+    <row r="112" ht="43.5" customHeight="1" s="46">
+      <c r="C112" s="23" t="inlineStr">
         <is>
           <t>time(s)</t>
         </is>
       </c>
-      <c r="D111" s="42" t="inlineStr">
+      <c r="D112" s="42" t="inlineStr">
         <is>
           <t>Description</t>
-        </is>
-      </c>
-      <c r="E111" s="60" t="n"/>
-      <c r="F111" s="60" t="n"/>
-      <c r="G111" s="60" t="n"/>
-      <c r="H111" s="60" t="n"/>
-      <c r="I111" s="60" t="n"/>
-      <c r="J111" s="60" t="n"/>
-      <c r="K111" s="60" t="n"/>
-      <c r="L111" s="60" t="n"/>
-      <c r="M111" s="60" t="n"/>
-      <c r="N111" s="59" t="n"/>
-    </row>
-    <row r="112" ht="43.5" customHeight="1" s="46">
-      <c r="C112" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="D112" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> - When a quest objective is visible on the minimap, display an arrow above the quest icon. See the image on the right.
- - When the character and quest objective are in the same zone but the quest point is NOT visible on the minimap, display a directional effect pointing toward the target.
- - When the character and quest objective are in different zones, display a directional effect pointing toward the nearest warp gimmick that leads to that zone.</t>
         </is>
       </c>
       <c r="E112" s="60" t="n"/>
@@ -2533,13 +2537,14 @@
       <c r="N112" s="59" t="n"/>
     </row>
     <row r="113" ht="29.25" customHeight="1" s="46">
-      <c r="C113" s="24" t="n">
-        <v>2</v>
-      </c>
-      <c r="D113" s="42" t="inlineStr">
-        <is>
-          <t>- Icon displayed at quest display condition point
-    - Tracked quest highlighted with border</t>
+      <c r="C113" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D113" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> - When a quest objective is visible on the minimap, display an arrow above the quest icon. See the image on the right.
+ - When the character and quest objective are in the same zone but the quest point is NOT visible on the minimap, display a directional effect pointing toward the target.
+ - When the character and quest objective are in different zones, display a directional effect pointing toward the nearest warp gimmick that leads to that zone.</t>
         </is>
       </c>
       <c r="E113" s="60" t="n"/>
@@ -2555,11 +2560,12 @@
     </row>
     <row r="114" ht="52.5" customHeight="1" s="46">
       <c r="C114" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D114" s="42" t="inlineStr">
         <is>
-          <t>- Glowing inverted triangle displayed above quest monster on minimap</t>
+          <t>- Icon displayed at quest display condition point
+    - Tracked quest highlighted with border</t>
         </is>
       </c>
       <c r="E114" s="60" t="n"/>
@@ -2573,8 +2579,28 @@
       <c r="M114" s="60" t="n"/>
       <c r="N114" s="59" t="n"/>
     </row>
+    <row r="115">
+      <c r="C115" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D115" s="42" t="inlineStr">
+        <is>
+          <t>- Glowing inverted triangle displayed above quest monster on minimap</t>
+        </is>
+      </c>
+      <c r="E115" s="60" t="n"/>
+      <c r="F115" s="60" t="n"/>
+      <c r="G115" s="60" t="n"/>
+      <c r="H115" s="60" t="n"/>
+      <c r="I115" s="60" t="n"/>
+      <c r="J115" s="60" t="n"/>
+      <c r="K115" s="60" t="n"/>
+      <c r="L115" s="60" t="n"/>
+      <c r="M115" s="60" t="n"/>
+      <c r="N115" s="59" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="30">
     <mergeCell ref="D69:N69"/>
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="H13:N13"/>
@@ -2601,6 +2627,7 @@
     <mergeCell ref="D114:N114"/>
     <mergeCell ref="D42:K42"/>
     <mergeCell ref="H11:N11"/>
+    <mergeCell ref="A1:O1"/>
     <mergeCell ref="D113:N113"/>
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="H16:N16"/>

</xml_diff>

<commit_message>
Fix XLSX translation quality + restore UI images + fix doc history rows
- Restore original UI wireframe images in Records/Codex (revert blur masking)
- Fix document history sheet row shifts (restore original structure)
- Translate 문서_히스토리 content entries to natural English
- Fix 144+ broken translations in World (Dimensional Gate, Time Gate, zone names)
- Fix Exploration Mission System garbled UI descriptions
- Fix Achievements, Adventure Journal, Constellation of Bonds UI text
- Fix Quest Guide System broken toggle descriptions
- Fix Codex Monster banner navigation typo

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QuestGuide_DesignDocument.xlsx
+++ b/docs/QuestGuide_DesignDocument.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="16">
     <font>
       <name val="맑은 고딕"/>
       <charset val="129"/>
@@ -139,15 +139,8 @@
       <name val="맑은 고딕"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <i val="1"/>
-      <color rgb="00CC0000"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -166,12 +159,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2F2"/>
-        <bgColor rgb="00FFF2F2"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="43">
     <border>
@@ -705,7 +692,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -889,9 +876,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1557,7 +1541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A2:L42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="4.375" customWidth="1" style="32" min="1" max="1"/>
@@ -1569,116 +1553,109 @@
     <col width="9" customWidth="1" style="32" min="17" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1" s="46">
-      <c r="A1" s="70" t="inlineStr">
-        <is>
-          <t>CONFIDENTIAL — Shared for portfolio review purposes only. All game content is the property of its respective studio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1" s="46"/>
+    <row r="2" ht="22" customHeight="1" s="46">
+      <c r="B2" s="61" t="inlineStr">
+        <is>
+          <t>Document History : Quest Guide System</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n"/>
+      <c r="D2" s="5" t="n"/>
+      <c r="E2" s="5" t="n"/>
+      <c r="F2" s="5" t="n"/>
+      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="5" t="n"/>
+      <c r="I2" s="5" t="n"/>
+      <c r="J2" s="5" t="n"/>
+      <c r="K2" s="5" t="n"/>
+      <c r="L2" s="5" t="n"/>
+    </row>
     <row r="3" ht="18" customHeight="1" s="46">
-      <c r="B3" s="61" t="inlineStr">
-        <is>
-          <t>Document History : Quest Guide System</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
-      <c r="K3" s="5" t="n"/>
-      <c r="L3" s="5" t="n"/>
+      <c r="B3" s="62" t="n"/>
+      <c r="C3" s="62" t="n"/>
+      <c r="D3" s="62" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="n"/>
+      <c r="K3" s="6" t="n"/>
+      <c r="L3" s="62" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1" s="46">
-      <c r="B4" s="62" t="inlineStr">
+      <c r="A4" s="7" t="n"/>
+      <c r="B4" s="63" t="inlineStr">
         <is>
           <t>Index</t>
         </is>
       </c>
-      <c r="C4" s="62" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="D4" s="62" t="inlineStr">
+      <c r="C4" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Date</t>
+        </is>
+      </c>
+      <c r="D4" s="64" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="L4" s="65" t="inlineStr">
         <is>
           <t>Author</t>
         </is>
       </c>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="n"/>
-      <c r="K4" s="6" t="n"/>
-      <c r="L4" s="62" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1" s="46">
-      <c r="A5" s="7" t="n"/>
-      <c r="B5" s="63" t="n">
+      <c r="A5" s="30" t="n"/>
+      <c r="B5" s="66" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="64" t="inlineStr">
+      <c r="C5" s="67" t="inlineStr">
         <is>
           <t>24.05.03</t>
         </is>
       </c>
-      <c r="D5" s="64" t="inlineStr">
+      <c r="D5" s="68" t="inlineStr">
         <is>
           <t>Initial draft</t>
         </is>
       </c>
-      <c r="E5" s="0" t="inlineStr">
+      <c r="L5" s="69" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
-      <c r="L5" s="65" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="30" t="n"/>
-      <c r="B6" s="66" t="n">
+      <c r="B6" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="67" t="inlineStr">
+      <c r="C6" s="28" t="inlineStr">
         <is>
           <t>25.06.11</t>
         </is>
       </c>
-      <c r="D6" s="68" t="inlineStr">
+      <c r="D6" s="52" t="inlineStr">
         <is>
           <t>UI updated; detailed descriptions added</t>
         </is>
       </c>
-      <c r="E6" s="0" t="inlineStr">
+      <c r="L6" s="27" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
-      <c r="L6" s="69" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="30" t="n"/>
-      <c r="B7" s="31" t="n"/>
-      <c r="C7" s="28" t="n"/>
-      <c r="D7" s="52" t="n"/>
-      <c r="L7" s="27" t="n"/>
+      <c r="B7" s="40" t="n"/>
+      <c r="C7" s="40" t="n"/>
+      <c r="D7" s="40" t="n"/>
+      <c r="L7" s="40" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="40" t="n"/>
-      <c r="C8" s="40" t="n"/>
-      <c r="D8" s="40" t="n"/>
-      <c r="L8" s="40" t="n"/>
+      <c r="D8" s="32" t="n"/>
     </row>
     <row r="9">
       <c r="D9" s="32" t="n"/>
@@ -1704,8 +1681,8 @@
     <row r="16">
       <c r="D16" s="32" t="n"/>
     </row>
-    <row r="17">
-      <c r="D17" s="32" t="n"/>
+    <row r="31">
+      <c r="D31" s="32" t="n"/>
     </row>
     <row r="32">
       <c r="D32" s="32" t="n"/>
@@ -1740,13 +1717,7 @@
     <row r="42">
       <c r="D42" s="32" t="n"/>
     </row>
-    <row r="43">
-      <c r="D43" s="32" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" verticalDpi="0"/>
 </worksheet>
@@ -1758,7 +1729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O115"/>
+  <dimension ref="A1:O114"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="16.5"/>
   <cols>
     <col width="2.625" customWidth="1" style="1" min="1" max="1"/>
@@ -1771,88 +1742,118 @@
     <col width="8.625" customWidth="1" style="1" min="9" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1" s="46">
-      <c r="A1" s="70" t="inlineStr">
-        <is>
-          <t>CONFIDENTIAL — Shared for portfolio review purposes only. All game content is the property of its respective studio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="27.95" customHeight="1" s="46"/>
-    <row r="3" s="46">
-      <c r="B3" s="18" t="inlineStr">
+    <row r="1" ht="3.95" customHeight="1" s="46"/>
+    <row r="2" ht="27.95" customHeight="1" s="46">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Quest Guide System</t>
         </is>
       </c>
-      <c r="C3" s="18" t="n"/>
-      <c r="D3" s="18" t="n"/>
-      <c r="E3" s="18" t="n"/>
-      <c r="F3" s="18" t="n"/>
-      <c r="G3" s="18" t="n"/>
-      <c r="H3" s="18" t="n"/>
-      <c r="I3" s="18" t="n"/>
-      <c r="J3" s="18" t="n"/>
-      <c r="K3" s="18" t="n"/>
-      <c r="L3" s="18" t="n"/>
-      <c r="M3" s="18" t="n"/>
-      <c r="N3" s="18" t="n"/>
-      <c r="O3" s="18" t="n"/>
-    </row>
-    <row r="4" ht="17.25" customHeight="1" s="46"/>
+      <c r="C2" s="18" t="n"/>
+      <c r="D2" s="18" t="n"/>
+      <c r="E2" s="18" t="n"/>
+      <c r="F2" s="18" t="n"/>
+      <c r="G2" s="18" t="n"/>
+      <c r="H2" s="18" t="n"/>
+      <c r="I2" s="18" t="n"/>
+      <c r="J2" s="18" t="n"/>
+      <c r="K2" s="18" t="n"/>
+      <c r="L2" s="18" t="n"/>
+      <c r="M2" s="18" t="n"/>
+      <c r="N2" s="18" t="n"/>
+      <c r="O2" s="18" t="n"/>
+    </row>
+    <row r="3" s="46"/>
+    <row r="4" ht="17.25" customHeight="1" s="46">
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Design Intent</t>
+        </is>
+      </c>
+    </row>
     <row r="5" s="46">
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>Design Intent</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" s="46">
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>- Provides convenience for quest location and direction</t>
         </is>
       </c>
     </row>
-    <row r="7" s="46"/>
+    <row r="6" s="46"/>
+    <row r="7" s="46">
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Display by Unit</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="20" t="n"/>
+      <c r="G7" s="20" t="n"/>
+      <c r="H7" s="20" t="n"/>
+      <c r="I7" s="21" t="n"/>
+      <c r="J7" s="21" t="n"/>
+      <c r="K7" s="21" t="n"/>
+      <c r="L7" s="21" t="n"/>
+      <c r="M7" s="21" t="n"/>
+      <c r="N7" s="21" t="n"/>
+    </row>
     <row r="8" ht="35.25" customHeight="1" s="46">
-      <c r="C8" s="15" t="inlineStr">
-        <is>
-          <t>Display by Unit</t>
-        </is>
-      </c>
-      <c r="E8" s="21" t="n"/>
-      <c r="F8" s="20" t="n"/>
-      <c r="G8" s="20" t="n"/>
-      <c r="H8" s="20" t="n"/>
+      <c r="C8" s="41" t="inlineStr">
+        <is>
+          <t>Quest Condition</t>
+        </is>
+      </c>
+      <c r="D8" s="59" t="n"/>
+      <c r="E8" s="41" t="inlineStr">
+        <is>
+          <t>Navigation Guide</t>
+        </is>
+      </c>
+      <c r="F8" s="41" t="inlineStr">
+        <is>
+          <t>Guide Effect</t>
+        </is>
+      </c>
+      <c r="G8" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="H8" s="41" t="inlineStr">
+        <is>
+          <t>Special Notes</t>
+        </is>
+      </c>
+      <c r="I8" s="60" t="n"/>
+      <c r="J8" s="60" t="n"/>
+      <c r="K8" s="60" t="n"/>
+      <c r="L8" s="60" t="n"/>
+      <c r="M8" s="60" t="n"/>
+      <c r="N8" s="59" t="n"/>
     </row>
     <row r="9" ht="31.5" customHeight="1" s="46">
-      <c r="C9" s="41" t="inlineStr">
-        <is>
-          <t>Quest Condition</t>
+      <c r="C9" s="43" t="inlineStr">
+        <is>
+          <t>CondTutorial</t>
         </is>
       </c>
       <c r="D9" s="59" t="n"/>
-      <c r="E9" s="41" t="inlineStr">
-        <is>
-          <t>Navigation Guide</t>
-        </is>
-      </c>
-      <c r="F9" s="41" t="inlineStr">
-        <is>
-          <t>Guide Effect</t>
-        </is>
-      </c>
-      <c r="G9" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="H9" s="41" t="inlineStr">
-        <is>
-          <t>Special Notes</t>
-        </is>
-      </c>
+      <c r="E9" s="43" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F9" s="43" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G9" s="43" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H9" s="43" t="n"/>
       <c r="I9" s="60" t="n"/>
       <c r="J9" s="60" t="n"/>
       <c r="K9" s="60" t="n"/>
@@ -1863,23 +1864,23 @@
     <row r="10" ht="31.5" customHeight="1" s="46">
       <c r="C10" s="43" t="inlineStr">
         <is>
-          <t>CondTutorial</t>
+          <t>CondDialog</t>
         </is>
       </c>
       <c r="D10" s="59" t="n"/>
       <c r="E10" s="43" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="F10" s="43" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="G10" s="43" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="H10" s="43" t="n"/>
@@ -1893,7 +1894,7 @@
     <row r="11" ht="34.5" customHeight="1" s="46">
       <c r="C11" s="43" t="inlineStr">
         <is>
-          <t>CondDialog</t>
+          <t>CondMonster</t>
         </is>
       </c>
       <c r="D11" s="59" t="n"/>
@@ -1912,7 +1913,12 @@
           <t>O</t>
         </is>
       </c>
-      <c r="H11" s="43" t="n"/>
+      <c r="H11" s="43" t="inlineStr">
+        <is>
+          <t>• Guide effect displayed above target monster's head
+• Navigation guide displayed only in areas where the quest monster is not placed</t>
+        </is>
+      </c>
       <c r="I11" s="60" t="n"/>
       <c r="J11" s="60" t="n"/>
       <c r="K11" s="60" t="n"/>
@@ -1923,7 +1929,7 @@
     <row r="12" ht="44.25" customHeight="1" s="46">
       <c r="C12" s="43" t="inlineStr">
         <is>
-          <t>CondMonster</t>
+          <t>CondItem</t>
         </is>
       </c>
       <c r="D12" s="59" t="n"/>
@@ -1944,8 +1950,8 @@
       </c>
       <c r="H12" s="43" t="inlineStr">
         <is>
-          <t>• Guide effect displayed above target monster's head
-• Navigation guide displayed only in areas where the quest monster is not placed</t>
+          <t>• Guide effect displayed above monsters that drop target items
+• Navigation guide displayed only in areas where item-dropping monsters are not placed</t>
         </is>
       </c>
       <c r="I12" s="60" t="n"/>
@@ -1958,7 +1964,7 @@
     <row r="13" ht="24" customHeight="1" s="46">
       <c r="C13" s="43" t="inlineStr">
         <is>
-          <t>CondItem</t>
+          <t>CondCutscene</t>
         </is>
       </c>
       <c r="D13" s="59" t="n"/>
@@ -1977,12 +1983,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="H13" s="43" t="inlineStr">
-        <is>
-          <t>• Guide effect displayed above monsters that drop target items
-• Navigation guide displayed only in areas where item-dropping monsters are not placed</t>
-        </is>
-      </c>
+      <c r="H13" s="43" t="n"/>
       <c r="I13" s="60" t="n"/>
       <c r="J13" s="60" t="n"/>
       <c r="K13" s="60" t="n"/>
@@ -1993,7 +1994,7 @@
     <row r="14" ht="21.75" customHeight="1" s="46">
       <c r="C14" s="43" t="inlineStr">
         <is>
-          <t>CondCutscene</t>
+          <t>CondArea</t>
         </is>
       </c>
       <c r="D14" s="59" t="n"/>
@@ -2023,7 +2024,7 @@
     <row r="15" ht="46.5" customHeight="1" s="46">
       <c r="C15" s="43" t="inlineStr">
         <is>
-          <t>CondArea</t>
+          <t>CondGimmick</t>
         </is>
       </c>
       <c r="D15" s="59" t="n"/>
@@ -2042,7 +2043,13 @@
           <t>O</t>
         </is>
       </c>
-      <c r="H15" s="43" t="n"/>
+      <c r="H15" s="43" t="inlineStr">
+        <is>
+          <t>• When multiple quest gimmicks are targets
+    ◦ Guide effect displayed for all gimmicks
+    ◦ Navigation guide displayed only in areas without those gimmicks</t>
+        </is>
+      </c>
       <c r="I15" s="60" t="n"/>
       <c r="J15" s="60" t="n"/>
       <c r="K15" s="60" t="n"/>
@@ -2053,7 +2060,7 @@
     <row r="16" ht="21.75" customHeight="1" s="46">
       <c r="C16" s="43" t="inlineStr">
         <is>
-          <t>CondGimmick</t>
+          <t>CondIndun</t>
         </is>
       </c>
       <c r="D16" s="59" t="n"/>
@@ -2074,9 +2081,7 @@
       </c>
       <c r="H16" s="43" t="inlineStr">
         <is>
-          <t>• When multiple quest gimmicks are targets
-    ◦ Guide effect displayed for all gimmicks
-    ◦ Navigation guide displayed only in areas without those gimmicks</t>
+          <t>• Gimmick allowing entry to the Instance Dungeon marked as target</t>
         </is>
       </c>
       <c r="I16" s="60" t="n"/>
@@ -2087,55 +2092,24 @@
       <c r="N16" s="59" t="n"/>
     </row>
     <row r="17" s="46">
-      <c r="C17" s="43" t="inlineStr">
-        <is>
-          <t>CondIndun</t>
-        </is>
-      </c>
-      <c r="D17" s="59" t="n"/>
-      <c r="E17" s="43" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="F17" s="43" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="G17" s="43" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="H17" s="43" t="inlineStr">
-        <is>
-          <t>• Gimmick allowing entry to the Instance Dungeon marked as target</t>
-        </is>
-      </c>
-      <c r="I17" s="60" t="n"/>
-      <c r="J17" s="60" t="n"/>
-      <c r="K17" s="60" t="n"/>
-      <c r="L17" s="60" t="n"/>
-      <c r="M17" s="60" t="n"/>
-      <c r="N17" s="59" t="n"/>
+      <c r="C17" s="14" t="n"/>
     </row>
     <row r="18" s="46">
-      <c r="C18" s="14" t="n"/>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>Quest Navigation Guide</t>
+        </is>
+      </c>
     </row>
     <row r="19" s="46">
-      <c r="C19" s="15" t="inlineStr">
-        <is>
-          <t>Quest Navigation Guide</t>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>- Arrow indicators around the character guide the quest destination</t>
         </is>
       </c>
     </row>
     <row r="20" s="46">
-      <c r="C20" s="26" t="inlineStr">
-        <is>
-          <t>- Arrow indicators around the character guide the quest destination</t>
-        </is>
-      </c>
+      <c r="C20" s="14" t="n"/>
     </row>
     <row r="21" s="46">
       <c r="C21" s="14" t="n"/>
@@ -2198,17 +2172,31 @@
       <c r="C40" s="14" t="n"/>
     </row>
     <row r="41" ht="17.25" customHeight="1" s="46">
-      <c r="C41" s="14" t="n"/>
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>time(s)</t>
+        </is>
+      </c>
+      <c r="D41" s="45" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E41" s="60" t="n"/>
+      <c r="F41" s="60" t="n"/>
+      <c r="G41" s="60" t="n"/>
+      <c r="H41" s="60" t="n"/>
+      <c r="I41" s="60" t="n"/>
+      <c r="J41" s="60" t="n"/>
+      <c r="K41" s="59" t="n"/>
     </row>
     <row r="42" ht="84.75" customHeight="1" s="46">
-      <c r="C42" s="17" t="inlineStr">
-        <is>
-          <t>time(s)</t>
-        </is>
-      </c>
-      <c r="D42" s="45" t="inlineStr">
-        <is>
-          <t>Description</t>
+      <c r="C42" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="42" t="inlineStr">
+        <is>
+          <t>- On click, toggle quest guide direction display on/off</t>
         </is>
       </c>
       <c r="E42" s="60" t="n"/>
@@ -2221,16 +2209,11 @@
     </row>
     <row r="43" ht="62.25" customHeight="1" s="46">
       <c r="C43" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D43" s="42" t="inlineStr">
         <is>
-          <t>My Display On/Off Button
-- Click when, Quest Guide Direction Display, Not Display before
- → Display during state in Click when, Not Display
- → Not Display during state in Click when, Display
-- Display state in Corresponding Icon Color to Display
-- Not Display state in Corresponding Icon Greyscale processing</t>
+          <t>- Quest Guide shows directional arrow around character. Arrow periodically points toward objective.</t>
         </is>
       </c>
       <c r="E43" s="60" t="n"/>
@@ -2242,38 +2225,24 @@
       <c r="K43" s="59" t="n"/>
     </row>
     <row r="44" s="46">
-      <c r="C44" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="D44" s="42" t="inlineStr">
-        <is>
-          <t>Quest Guide effect displayed arrow displayed. arrow periodically - move possible ‘’ defeat , Quest Monster placement zone PC displayed gimmick placement zone PC displayed - cutscene displayed</t>
-        </is>
-      </c>
-      <c r="E44" s="60" t="n"/>
-      <c r="F44" s="60" t="n"/>
-      <c r="G44" s="60" t="n"/>
-      <c r="H44" s="60" t="n"/>
-      <c r="I44" s="60" t="n"/>
-      <c r="J44" s="60" t="n"/>
-      <c r="K44" s="59" t="n"/>
+      <c r="C44" s="14" t="n"/>
     </row>
     <row r="45" s="46">
-      <c r="C45" s="14" t="n"/>
+      <c r="C45" s="15" t="inlineStr">
+        <is>
+          <t>Guide Effect</t>
+        </is>
+      </c>
     </row>
     <row r="46" s="46">
-      <c r="C46" s="15" t="inlineStr">
-        <is>
-          <t>Guide Effect</t>
+      <c r="C46" s="26" t="inlineStr">
+        <is>
+          <t>- Effect directly marking the quest objective</t>
         </is>
       </c>
     </row>
     <row r="47" s="46">
-      <c r="C47" s="26" t="inlineStr">
-        <is>
-          <t>- Effect directly marking the quest objective</t>
-        </is>
-      </c>
+      <c r="C47" s="14" t="n"/>
     </row>
     <row r="48" s="46">
       <c r="C48" s="14" t="n"/>
@@ -2339,17 +2308,34 @@
       <c r="C68" s="14" t="n"/>
     </row>
     <row r="69" s="46">
-      <c r="C69" s="14" t="n"/>
+      <c r="C69" s="23" t="inlineStr">
+        <is>
+          <t>time(s)</t>
+        </is>
+      </c>
+      <c r="D69" s="42" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E69" s="60" t="n"/>
+      <c r="F69" s="60" t="n"/>
+      <c r="G69" s="60" t="n"/>
+      <c r="H69" s="60" t="n"/>
+      <c r="I69" s="60" t="n"/>
+      <c r="J69" s="60" t="n"/>
+      <c r="K69" s="60" t="n"/>
+      <c r="L69" s="60" t="n"/>
+      <c r="M69" s="60" t="n"/>
+      <c r="N69" s="59" t="n"/>
     </row>
     <row r="70" ht="16.5" customHeight="1" s="46">
-      <c r="C70" s="23" t="inlineStr">
-        <is>
-          <t>time(s)</t>
-        </is>
+      <c r="C70" s="23" t="n">
+        <v>1</v>
       </c>
       <c r="D70" s="42" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Location guide for specific points, NPCs, gimmick objects</t>
         </is>
       </c>
       <c r="E70" s="60" t="n"/>
@@ -2364,32 +2350,12 @@
       <c r="N70" s="59" t="n"/>
     </row>
     <row r="71" ht="210.75" customHeight="1" s="46">
-      <c r="C71" s="23" t="n">
-        <v>1</v>
+      <c r="C71" s="24" t="inlineStr">
+        <is>
+          <t>Display Conditions</t>
+        </is>
       </c>
       <c r="D71" s="42" t="inlineStr">
-        <is>
-          <t>Location guide for specific points, NPCs, gimmick objects</t>
-        </is>
-      </c>
-      <c r="E71" s="60" t="n"/>
-      <c r="F71" s="60" t="n"/>
-      <c r="G71" s="60" t="n"/>
-      <c r="H71" s="60" t="n"/>
-      <c r="I71" s="60" t="n"/>
-      <c r="J71" s="60" t="n"/>
-      <c r="K71" s="60" t="n"/>
-      <c r="L71" s="60" t="n"/>
-      <c r="M71" s="60" t="n"/>
-      <c r="N71" s="59" t="n"/>
-    </row>
-    <row r="72" ht="46.5" customHeight="1" s="46">
-      <c r="C72" s="24" t="inlineStr">
-        <is>
-          <t>Display Conditions</t>
-        </is>
-      </c>
-      <c r="D72" s="42" t="inlineStr">
         <is>
           <t>in progress 
 - QuestMissionList status list
@@ -2409,6 +2375,30 @@
 - cutscene displayed</t>
         </is>
       </c>
+      <c r="E71" s="60" t="n"/>
+      <c r="F71" s="60" t="n"/>
+      <c r="G71" s="60" t="n"/>
+      <c r="H71" s="60" t="n"/>
+      <c r="I71" s="60" t="n"/>
+      <c r="J71" s="60" t="n"/>
+      <c r="K71" s="60" t="n"/>
+      <c r="L71" s="60" t="n"/>
+      <c r="M71" s="60" t="n"/>
+      <c r="N71" s="59" t="n"/>
+    </row>
+    <row r="72" ht="46.5" customHeight="1" s="46">
+      <c r="C72" s="24" t="inlineStr">
+        <is>
+          <t>Quest Effect</t>
+        </is>
+      </c>
+      <c r="D72" s="42" t="inlineStr">
+        <is>
+          <t>- Effect names
+    ◦ QuestCompleteLoop01
+    ◦ QuestCompleteShot01</t>
+        </is>
+      </c>
       <c r="E72" s="60" t="n"/>
       <c r="F72" s="60" t="n"/>
       <c r="G72" s="60" t="n"/>
@@ -2421,45 +2411,24 @@
       <c r="N72" s="59" t="n"/>
     </row>
     <row r="73" s="46">
-      <c r="C73" s="24" t="inlineStr">
-        <is>
-          <t>Quest Effect</t>
-        </is>
-      </c>
-      <c r="D73" s="42" t="inlineStr">
-        <is>
-          <t>- Effect names
-    ◦ QuestCompleteLoop01
-    ◦ QuestCompleteShot01</t>
-        </is>
-      </c>
-      <c r="E73" s="60" t="n"/>
-      <c r="F73" s="60" t="n"/>
-      <c r="G73" s="60" t="n"/>
-      <c r="H73" s="60" t="n"/>
-      <c r="I73" s="60" t="n"/>
-      <c r="J73" s="60" t="n"/>
-      <c r="K73" s="60" t="n"/>
-      <c r="L73" s="60" t="n"/>
-      <c r="M73" s="60" t="n"/>
-      <c r="N73" s="59" t="n"/>
+      <c r="C73" s="14" t="n"/>
     </row>
     <row r="74" s="46">
-      <c r="C74" s="14" t="n"/>
+      <c r="C74" s="15" t="inlineStr">
+        <is>
+          <t>Quest Monster Guide</t>
+        </is>
+      </c>
     </row>
     <row r="75" s="46">
-      <c r="C75" s="15" t="inlineStr">
-        <is>
-          <t>Quest Monster Guide</t>
+      <c r="C75" s="25" t="inlineStr">
+        <is>
+          <t>- Exclamation mark displayed above monster's head</t>
         </is>
       </c>
     </row>
     <row r="76" s="46">
-      <c r="C76" s="25" t="inlineStr">
-        <is>
-          <t>- Exclamation mark displayed above monster's head</t>
-        </is>
-      </c>
+      <c r="C76" s="14" t="n"/>
     </row>
     <row r="77" s="46">
       <c r="C77" s="14" t="n"/>
@@ -2476,9 +2445,7 @@
     <row r="81" s="46">
       <c r="C81" s="14" t="n"/>
     </row>
-    <row r="82" s="46">
-      <c r="C82" s="14" t="n"/>
-    </row>
+    <row r="82" s="46"/>
     <row r="83" s="46"/>
     <row r="84" s="46"/>
     <row r="85" s="46"/>
@@ -2489,14 +2456,14 @@
     <row r="90" s="46"/>
     <row r="91" s="46"/>
     <row r="92" s="46"/>
-    <row r="93" s="46"/>
-    <row r="94" s="46">
-      <c r="C94" s="15" t="inlineStr">
+    <row r="93" s="46">
+      <c r="C93" s="15" t="inlineStr">
         <is>
           <t>Minimap Marking</t>
         </is>
       </c>
     </row>
+    <row r="94" s="46"/>
     <row r="95" s="46"/>
     <row r="96" s="46"/>
     <row r="97" s="46"/>
@@ -2513,16 +2480,37 @@
     <row r="108" s="46"/>
     <row r="109" s="46"/>
     <row r="110" s="46"/>
-    <row r="111" s="46"/>
+    <row r="111" s="46">
+      <c r="C111" s="23" t="inlineStr">
+        <is>
+          <t>time(s)</t>
+        </is>
+      </c>
+      <c r="D111" s="42" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E111" s="60" t="n"/>
+      <c r="F111" s="60" t="n"/>
+      <c r="G111" s="60" t="n"/>
+      <c r="H111" s="60" t="n"/>
+      <c r="I111" s="60" t="n"/>
+      <c r="J111" s="60" t="n"/>
+      <c r="K111" s="60" t="n"/>
+      <c r="L111" s="60" t="n"/>
+      <c r="M111" s="60" t="n"/>
+      <c r="N111" s="59" t="n"/>
+    </row>
     <row r="112" ht="43.5" customHeight="1" s="46">
-      <c r="C112" s="23" t="inlineStr">
-        <is>
-          <t>time(s)</t>
-        </is>
-      </c>
-      <c r="D112" s="42" t="inlineStr">
-        <is>
-          <t>Description</t>
+      <c r="C112" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D112" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> - When a quest objective is visible on the minimap, display an arrow above the quest icon. See the image on the right.
+ - When the character and quest objective are in the same zone but the quest point is NOT visible on the minimap, display a directional effect pointing toward the target.
+ - When the character and quest objective are in different zones, display a directional effect pointing toward the nearest warp gimmick that leads to that zone.</t>
         </is>
       </c>
       <c r="E112" s="60" t="n"/>
@@ -2537,14 +2525,13 @@
       <c r="N112" s="59" t="n"/>
     </row>
     <row r="113" ht="29.25" customHeight="1" s="46">
-      <c r="C113" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="D113" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> - When a quest objective is visible on the minimap, display an arrow above the quest icon. See the image on the right.
- - When the character and quest objective are in the same zone but the quest point is NOT visible on the minimap, display a directional effect pointing toward the target.
- - When the character and quest objective are in different zones, display a directional effect pointing toward the nearest warp gimmick that leads to that zone.</t>
+      <c r="C113" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D113" s="42" t="inlineStr">
+        <is>
+          <t>- Icon displayed at quest display condition point
+    - Tracked quest highlighted with border</t>
         </is>
       </c>
       <c r="E113" s="60" t="n"/>
@@ -2560,12 +2547,11 @@
     </row>
     <row r="114" ht="52.5" customHeight="1" s="46">
       <c r="C114" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D114" s="42" t="inlineStr">
         <is>
-          <t>- Icon displayed at quest display condition point
-    - Tracked quest highlighted with border</t>
+          <t>- Glowing inverted triangle displayed above quest monster on minimap</t>
         </is>
       </c>
       <c r="E114" s="60" t="n"/>
@@ -2579,28 +2565,8 @@
       <c r="M114" s="60" t="n"/>
       <c r="N114" s="59" t="n"/>
     </row>
-    <row r="115">
-      <c r="C115" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="D115" s="42" t="inlineStr">
-        <is>
-          <t>- Glowing inverted triangle displayed above quest monster on minimap</t>
-        </is>
-      </c>
-      <c r="E115" s="60" t="n"/>
-      <c r="F115" s="60" t="n"/>
-      <c r="G115" s="60" t="n"/>
-      <c r="H115" s="60" t="n"/>
-      <c r="I115" s="60" t="n"/>
-      <c r="J115" s="60" t="n"/>
-      <c r="K115" s="60" t="n"/>
-      <c r="L115" s="60" t="n"/>
-      <c r="M115" s="60" t="n"/>
-      <c r="N115" s="59" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="29">
     <mergeCell ref="D69:N69"/>
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="H13:N13"/>
@@ -2627,7 +2593,6 @@
     <mergeCell ref="D114:N114"/>
     <mergeCell ref="D42:K42"/>
     <mergeCell ref="H11:N11"/>
-    <mergeCell ref="A1:O1"/>
     <mergeCell ref="D113:N113"/>
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="H16:N16"/>

</xml_diff>